<commit_message>
Extraer 36 preguntas reales del Excel a questions.json, actualizar areas a 6 y agrergar botones de Portal NyTEX a Landing
</commit_message>
<xml_diff>
--- a/Matriz del Diagnóstico Operativo - Consultores NyT.xlsx
+++ b/Matriz del Diagnóstico Operativo - Consultores NyT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emili\OneDrive\Desktop\Developer\Diagnóstico de preguntas revela fugas operativas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77DB5879-A87E-4104-BC47-15DBC8011B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D85467-5423-4ED2-AD43-18DA4488D1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{273E6615-ED72-484D-A321-61CCB6E33CF5}"/>
   </bookViews>
@@ -672,7 +672,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -733,6 +733,11 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -742,107 +747,11 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -904,47 +813,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -961,38 +840,38 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1336,7 +1215,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="34.799999999999997" x14ac:dyDescent="0.3">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1"/>
@@ -1345,7 +1224,7 @@
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="1"/>
@@ -1354,7 +1233,7 @@
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1"/>
@@ -1376,7 +1255,7 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="2:6" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="B7" s="20" t="s">
         <v>3</v>
       </c>
@@ -1386,7 +1265,7 @@
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="10" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="1"/>
@@ -1395,7 +1274,7 @@
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="11" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="1"/>
@@ -1404,7 +1283,7 @@
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="1"/>
@@ -1413,121 +1292,121 @@
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="14" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="16" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="F13" s="16" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="27" t="s">
+      <c r="F14" s="16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E15" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="27" t="s">
+      <c r="F15" s="16" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="16" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="16" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1545,8 +1424,8 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="2:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B20" s="3" t="s">
+    <row r="20" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B20" s="20" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="1"/>
@@ -1555,7 +1434,7 @@
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="1"/>
@@ -1564,7 +1443,7 @@
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C22" s="1"/>
@@ -1573,7 +1452,7 @@
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="2:6" ht="23.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>44</v>
       </c>
       <c r="C23" s="1"/>
@@ -1582,121 +1461,121 @@
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="D24" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="29" t="s">
+      <c r="E24" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F24" s="30" t="s">
+      <c r="F24" s="19" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B25" s="26" t="s">
+      <c r="B25" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="27" t="s">
+      <c r="C25" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="27" t="s">
+      <c r="D25" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="27" t="s">
+      <c r="E25" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="27" t="s">
+      <c r="F25" s="16" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="27" t="s">
+      <c r="D26" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="E26" s="27" t="s">
+      <c r="E26" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="F26" s="27" t="s">
+      <c r="F26" s="16" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="27" t="s">
+      <c r="C27" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="27" t="s">
+      <c r="D27" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="27" t="s">
+      <c r="E27" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F27" s="27" t="s">
+      <c r="F27" s="16" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="27" t="s">
+      <c r="D28" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="F28" s="27" t="s">
+      <c r="F28" s="16" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="26" t="s">
+      <c r="B29" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="27" t="s">
+      <c r="C29" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="27" t="s">
+      <c r="D29" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="E29" s="27" t="s">
+      <c r="E29" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="F29" s="27" t="s">
+      <c r="F29" s="16" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B30" s="26" t="s">
+      <c r="B30" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C30" s="27" t="s">
+      <c r="C30" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="27" t="s">
+      <c r="D30" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="E30" s="27" t="s">
+      <c r="E30" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F30" s="27" t="s">
+      <c r="F30" s="16" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1714,8 +1593,8 @@
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
     </row>
-    <row r="33" spans="2:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B33" s="3" t="s">
+    <row r="33" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B33" s="20" t="s">
         <v>74</v>
       </c>
       <c r="C33" s="1"/>
@@ -1724,7 +1603,7 @@
       <c r="F33" s="1"/>
     </row>
     <row r="34" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C34" s="1"/>
@@ -1733,7 +1612,7 @@
       <c r="F34" s="1"/>
     </row>
     <row r="35" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C35" s="1"/>
@@ -1741,8 +1620,8 @@
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B36" s="5" t="s">
+    <row r="36" spans="2:6" ht="23.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C36" s="1"/>
@@ -1750,122 +1629,122 @@
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
     </row>
-    <row r="37" spans="2:6" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="6" t="s">
+    <row r="37" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="B37" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="7" t="s">
+      <c r="E37" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F37" s="8" t="s">
+      <c r="F37" s="19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="9" t="s">
+    <row r="38" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B38" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="C38" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="F38" s="11" t="s">
+      <c r="F38" s="16" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="39" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="9" t="s">
+    <row r="39" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B39" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="F39" s="11" t="s">
+      <c r="F39" s="16" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="9" t="s">
+    <row r="40" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B40" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="E40" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="F40" s="16" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="9" t="s">
+    <row r="41" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B41" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="E41" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="F41" s="11" t="s">
+      <c r="F41" s="16" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="42" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="9" t="s">
+    <row r="42" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B42" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="E42" s="10" t="s">
+      <c r="E42" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="F42" s="11" t="s">
+      <c r="F42" s="16" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="43" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="C43" s="13" t="s">
+      <c r="C43" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="D43" s="13" t="s">
+      <c r="D43" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="F43" s="14" t="s">
+      <c r="F43" s="16" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1883,8 +1762,8 @@
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
     </row>
-    <row r="46" spans="2:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B46" s="3" t="s">
+    <row r="46" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B46" s="20" t="s">
         <v>107</v>
       </c>
       <c r="C46" s="1"/>
@@ -1893,7 +1772,7 @@
       <c r="F46" s="1"/>
     </row>
     <row r="47" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C47" s="1"/>
@@ -1902,7 +1781,7 @@
       <c r="F47" s="1"/>
     </row>
     <row r="48" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="4" t="s">
         <v>108</v>
       </c>
       <c r="C48" s="1"/>
@@ -1910,8 +1789,8 @@
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
     </row>
-    <row r="49" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B49" s="5" t="s">
+    <row r="49" spans="2:6" ht="23.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B49" s="4" t="s">
         <v>109</v>
       </c>
       <c r="C49" s="1"/>
@@ -1919,122 +1798,122 @@
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
     </row>
-    <row r="50" spans="2:6" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="6" t="s">
+    <row r="50" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="B50" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C50" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D50" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F50" s="8" t="s">
+      <c r="F50" s="19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="2:6" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B51" s="9" t="s">
+    <row r="51" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="B51" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E51" s="10" t="s">
+      <c r="E51" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="F51" s="11" t="s">
+      <c r="F51" s="16" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="52" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B52" s="9" t="s">
+    <row r="52" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B52" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="D52" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="E52" s="10" t="s">
+      <c r="E52" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="F52" s="11" t="s">
+      <c r="F52" s="16" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="53" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B53" s="9" t="s">
+    <row r="53" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B53" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="C53" s="10" t="s">
+      <c r="C53" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="D53" s="10" t="s">
+      <c r="D53" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="E53" s="10" t="s">
+      <c r="E53" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F53" s="11" t="s">
+      <c r="F53" s="16" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="54" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="9" t="s">
+    <row r="54" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B54" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="D54" s="10" t="s">
+      <c r="D54" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E54" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F54" s="11" t="s">
+      <c r="F54" s="16" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="55" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B55" s="9" t="s">
+    <row r="55" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B55" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="D55" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="E55" s="10" t="s">
+      <c r="E55" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="F55" s="11" t="s">
+      <c r="F55" s="16" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="56" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B56" s="12" t="s">
+      <c r="B56" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C56" s="13" t="s">
+      <c r="C56" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="D56" s="13" t="s">
+      <c r="D56" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="E56" s="13" t="s">
+      <c r="E56" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="F56" s="14" t="s">
+      <c r="F56" s="16" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2052,8 +1931,8 @@
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
     </row>
-    <row r="59" spans="2:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B59" s="3" t="s">
+    <row r="59" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B59" s="20" t="s">
         <v>140</v>
       </c>
       <c r="C59" s="1"/>
@@ -2062,7 +1941,7 @@
       <c r="F59" s="1"/>
     </row>
     <row r="60" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C60" s="1"/>
@@ -2071,7 +1950,7 @@
       <c r="F60" s="1"/>
     </row>
     <row r="61" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="4" t="s">
         <v>141</v>
       </c>
       <c r="C61" s="1"/>
@@ -2079,8 +1958,8 @@
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
     </row>
-    <row r="62" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B62" s="5" t="s">
+    <row r="62" spans="2:6" ht="23.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B62" s="4" t="s">
         <v>142</v>
       </c>
       <c r="C62" s="1"/>
@@ -2088,122 +1967,122 @@
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
     </row>
-    <row r="63" spans="2:6" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="6" t="s">
+    <row r="63" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="B63" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C63" s="7" t="s">
+      <c r="C63" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D63" s="7" t="s">
+      <c r="D63" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E63" s="7" t="s">
+      <c r="E63" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F63" s="8" t="s">
+      <c r="F63" s="19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B64" s="9" t="s">
+    <row r="64" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B64" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="D64" s="10" t="s">
+      <c r="D64" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="E64" s="10" t="s">
+      <c r="E64" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="F64" s="11" t="s">
+      <c r="F64" s="16" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="65" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B65" s="9" t="s">
+    <row r="65" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B65" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="C65" s="10" t="s">
+      <c r="C65" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="D65" s="10" t="s">
+      <c r="D65" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E65" s="10" t="s">
+      <c r="E65" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="F65" s="11" t="s">
+      <c r="F65" s="16" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="66" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B66" s="9" t="s">
+    <row r="66" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B66" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="C66" s="10" t="s">
+      <c r="C66" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="E66" s="10" t="s">
+      <c r="E66" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="F66" s="11" t="s">
+      <c r="F66" s="16" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="67" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="9" t="s">
+    <row r="67" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B67" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="C67" s="10" t="s">
+      <c r="C67" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="D67" s="10" t="s">
+      <c r="D67" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="E67" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="F67" s="11" t="s">
+      <c r="F67" s="16" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="68" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="9" t="s">
+    <row r="68" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B68" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="C68" s="10" t="s">
+      <c r="C68" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="D68" s="10" t="s">
+      <c r="D68" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="E68" s="10" t="s">
+      <c r="E68" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="F68" s="11" t="s">
+      <c r="F68" s="16" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="C69" s="13" t="s">
+      <c r="C69" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="D69" s="13" t="s">
+      <c r="D69" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="E69" s="13" t="s">
+      <c r="E69" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="F69" s="14" t="s">
+      <c r="F69" s="16" t="s">
         <v>172</v>
       </c>
     </row>
@@ -2221,8 +2100,8 @@
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
     </row>
-    <row r="72" spans="2:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="B72" s="3" t="s">
+    <row r="72" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B72" s="20" t="s">
         <v>173</v>
       </c>
       <c r="C72" s="1"/>
@@ -2231,7 +2110,7 @@
       <c r="F72" s="1"/>
     </row>
     <row r="73" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B73" s="4" t="s">
+      <c r="B73" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C73" s="1"/>
@@ -2240,7 +2119,7 @@
       <c r="F73" s="1"/>
     </row>
     <row r="74" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B74" s="5" t="s">
+      <c r="B74" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C74" s="1"/>
@@ -2248,8 +2127,8 @@
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
     </row>
-    <row r="75" spans="2:6" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="B75" s="5" t="s">
+    <row r="75" spans="2:6" ht="23.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B75" s="4" t="s">
         <v>175</v>
       </c>
       <c r="C75" s="1"/>
@@ -2257,127 +2136,127 @@
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
     </row>
-    <row r="76" spans="2:6" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B76" s="6" t="s">
+    <row r="76" spans="2:6" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="B76" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C76" s="7" t="s">
+      <c r="C76" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D76" s="7" t="s">
+      <c r="D76" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E76" s="7" t="s">
+      <c r="E76" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="F76" s="8" t="s">
+      <c r="F76" s="19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B77" s="9" t="s">
+    <row r="77" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B77" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="C77" s="10" t="s">
+      <c r="C77" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="D77" s="10" t="s">
+      <c r="D77" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="E77" s="10" t="s">
+      <c r="E77" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="F77" s="11" t="s">
+      <c r="F77" s="16" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="78" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B78" s="9" t="s">
+    <row r="78" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B78" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="C78" s="10" t="s">
+      <c r="C78" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="D78" s="10" t="s">
+      <c r="D78" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="E78" s="10" t="s">
+      <c r="E78" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="F78" s="11" t="s">
+      <c r="F78" s="16" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="79" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B79" s="9" t="s">
+    <row r="79" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B79" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="C79" s="10" t="s">
+      <c r="C79" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="D79" s="10" t="s">
+      <c r="D79" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="E79" s="10" t="s">
+      <c r="E79" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="F79" s="11" t="s">
+      <c r="F79" s="16" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="80" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B80" s="9" t="s">
+    <row r="80" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B80" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="C80" s="10" t="s">
+      <c r="C80" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="D80" s="10" t="s">
+      <c r="D80" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="E80" s="10" t="s">
+      <c r="E80" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="F80" s="11" t="s">
+      <c r="F80" s="16" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="81" spans="2:6" ht="51" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="9" t="s">
+    <row r="81" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="B81" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="C81" s="10" t="s">
+      <c r="C81" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="D81" s="10" t="s">
+      <c r="D81" s="16" t="s">
         <v>198</v>
       </c>
-      <c r="E81" s="10" t="s">
+      <c r="E81" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="F81" s="11" t="s">
+      <c r="F81" s="16" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="82" spans="2:6" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="B82" s="12" t="s">
+      <c r="B82" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="C82" s="13" t="s">
+      <c r="C82" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="D82" s="13" t="s">
+      <c r="D82" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="E82" s="13" t="s">
+      <c r="E82" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="F82" s="14" t="s">
+      <c r="F82" s="16" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="83" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B83" s="15" t="s">
+      <c r="B83" s="5" t="s">
         <v>206</v>
       </c>
       <c r="C83" s="1"/>
@@ -2386,7 +2265,7 @@
       <c r="F83" s="1"/>
     </row>
     <row r="84" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B84" s="16" t="s">
+      <c r="B84" s="6" t="s">
         <v>207</v>
       </c>
       <c r="C84" s="1"/>

</xml_diff>